<commit_message>
Ispravak greškice u bazi
</commit_message>
<xml_diff>
--- a/wc-data.xlsx
+++ b/wc-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c9d1b39c11dd659/Dokumenti/Apps/phc-stat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="652" documentId="8_{31E65144-C7D6-482C-BFB9-14E83E95C2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{304FED25-3186-4C9F-95F9-AA938F387331}"/>
+  <xr:revisionPtr revIDLastSave="653" documentId="8_{31E65144-C7D6-482C-BFB9-14E83E95C2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5EFEFF0-64D5-4B63-80A3-217DD52BDD4B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BABAC88A-431C-4718-AB57-202BD2B77C54}"/>
   </bookViews>
@@ -3033,6 +3033,9 @@
       <c r="J35" s="1">
         <v>4</v>
       </c>
+      <c r="K35" s="1">
+        <v>5</v>
+      </c>
       <c r="L35" s="1" t="s">
         <v>50</v>
       </c>

</xml_diff>